<commit_message>
Renommage Mapping CDA to FHIR (#66)
* Renommage Mapping CDA to FHIR

* Update input/fsh/MappingCDA_FHIR_Entete/PersonneStructureAssignedEntityFHIR.fsh

Co-authored-by: Nicolas Riss <48218773+nriss@users.noreply.github.com>

* Update input/fsh/MappingCDA_FHIR_Entete/PersonneStructureAuteurCDAFHIR.fsh

Co-authored-by: Nicolas Riss <48218773+nriss@users.noreply.github.com>

* Update input/fsh/MappingCDA_FHIR_Entete/PersonneStructureAuteurCDAFHIR.fsh

Co-authored-by: Nicolas Riss <48218773+nriss@users.noreply.github.com>

---------

Co-authored-by: Nicolas Riss <48218773+nriss@users.noreply.github.com> 8ff29b86bc42235c08cc25f4eb36a57ae5937f80
</commit_message>
<xml_diff>
--- a/main/ig/mappingAuteurCDAFHIR.xlsx
+++ b/main/ig/mappingAuteurCDAFHIR.xlsx
@@ -58,7 +58,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-21T15:23:03+00:00</t>
+    <t>2025-10-21T16:49:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -83,7 +83,7 @@
   </si>
   <si>
     <t xml:space="preserve">Ce ConceptMap présente deux groupes de mapping : 
- - Mapping 1 : entre le modèle métier \"auteur\" et l'élément CDA \"author\"
+ - Mapping 1 : entre le modèle métier \"Auteur\" et l'élément CDA \"author\"
  - Mapping 2 : entre l'élément CDA \"author\" et l'élément FHIR \"Composition.author\" </t>
   </si>
   <si>
@@ -105,16 +105,16 @@
     <t>Target</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/Auteur</t>
+    <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-auteur</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-core-author</t>
-  </si>
-  <si>
-    <t>Auteur</t>
+    <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-cda-author</t>
+  </si>
+  <si>
+    <t>FRLMAuteur</t>
   </si>
   <si>
     <t>equivalent</t>
@@ -123,25 +123,25 @@
     <t>author</t>
   </si>
   <si>
-    <t>Auteur.roleFonctionnel</t>
+    <t>FRLMAuteur.roleFonctionnel</t>
   </si>
   <si>
     <t>author.functionCode</t>
   </si>
   <si>
-    <t>Auteur.horodatageParticipation</t>
+    <t>FRLMAuteur.horodatageParticipation</t>
   </si>
   <si>
     <t>author.time</t>
   </si>
   <si>
-    <t>Auteur.PersonneStructure</t>
+    <t>FRLMAuteur.FRLMPersonneStructure</t>
   </si>
   <si>
     <t>author.assignedAuthor</t>
   </si>
   <si>
-    <t>Auteur.SystemeStructureAuteur</t>
+    <t>FRLMAuteur.FRLMSystemeStructureAuteur</t>
   </si>
   <si>
     <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-composition-document</t>

</xml_diff>